<commit_message>
Ad-hoc Credit Rating Monthly Analysis: 2026-09-01
</commit_message>
<xml_diff>
--- a/bqr/2026-10-01/_price.xlsx
+++ b/bqr/2026-10-01/_price.xlsx
@@ -486,22 +486,22 @@
         <v>28.47</v>
       </c>
       <c r="E2" t="n">
-        <v>27.93</v>
+        <v>27.935</v>
       </c>
       <c r="F2" t="n">
-        <v>28.235</v>
+        <v>28.17</v>
       </c>
       <c r="G2" t="n">
-        <v>1089285</v>
+        <v>1356913</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.195</v>
+        <v>-0.26</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.68589518</v>
+        <v>-0.91452691</v>
       </c>
       <c r="J2" t="n">
-        <v>28.21</v>
+        <v>28.19</v>
       </c>
     </row>
     <row r="3">

</xml_diff>